<commit_message>
Actualizar Excel seguimiento y notebook Pulmon Oriente v2
</commit_message>
<xml_diff>
--- a/ITT_Seguimiento_Datasets.xlsx
+++ b/ITT_Seguimiento_Datasets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge\Desktop\Itt_repos_cali\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A1BD2D5-0F41-419E-857A-E4568EFDCCE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAF79A16-A82C-4D99-8ACA-EE8A1B933EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Seguimiento Datasets" sheetId="1" r:id="rId1"/>
@@ -416,16 +416,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -458,6 +452,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -768,7 +771,7 @@
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" style="3" customWidth="1"/>
+    <col min="4" max="4" width="12" style="12" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
@@ -779,1362 +782,1362 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
     </row>
     <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K3" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="8" t="s">
+      <c r="G4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J4" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K4" s="8" t="s">
+      <c r="J4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="8" t="s">
+      <c r="G5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J5" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K5" s="8" t="s">
+      <c r="J5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="8" t="s">
+      <c r="G6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="I6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J6" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K6" s="8" t="s">
+      <c r="J6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H7" s="8" t="s">
+      <c r="G7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J7" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K7" s="8" t="s">
+      <c r="J7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" s="8" t="s">
+      <c r="G8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K8" s="8" t="s">
+      <c r="J8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K8" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="I9" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="J9" s="9" t="s">
+      <c r="J9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="K9" s="9" t="s">
+      <c r="K9" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I10" s="9" t="s">
+      <c r="I10" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="J10" s="9" t="s">
+      <c r="J10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="K10" s="9" t="s">
+      <c r="K10" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G11" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H11" s="8" t="s">
+      <c r="G11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="I11" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J11" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K11" s="8" t="s">
+      <c r="J11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G12" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H12" s="8" t="s">
+      <c r="G12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="8" t="s">
+      <c r="I12" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J12" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K12" s="8" t="s">
+      <c r="J12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K12" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I13" s="9" t="s">
+      <c r="I13" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="J13" s="9" t="s">
+      <c r="J13" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="K13" s="9" t="s">
+      <c r="K13" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G14" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H14" s="8" t="s">
+      <c r="G14" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I14" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J14" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K14" s="8" t="s">
+      <c r="J14" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K14" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H15" s="8" t="s">
+      <c r="G15" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="8" t="s">
+      <c r="I15" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J15" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K15" s="8" t="s">
+      <c r="J15" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K15" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G16" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H16" s="8" t="s">
+      <c r="G16" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H16" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="8" t="s">
+      <c r="I16" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J16" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K16" s="8" t="s">
+      <c r="J16" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K16" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G17" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H17" s="8" t="s">
+      <c r="G17" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="8" t="s">
+      <c r="I17" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J17" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K17" s="8" t="s">
+      <c r="J17" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K17" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G18" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H18" s="8" t="s">
+      <c r="G18" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="8" t="s">
+      <c r="I18" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J18" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K18" s="8" t="s">
+      <c r="J18" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K18" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I19" s="9" t="s">
+      <c r="I19" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="J19" s="9" t="s">
+      <c r="J19" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="K19" s="9" t="s">
+      <c r="K19" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="H20" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I20" s="9" t="s">
+      <c r="I20" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="J20" s="9" t="s">
+      <c r="J20" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="K20" s="9" t="s">
+      <c r="K20" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G21" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H21" s="8" t="s">
+      <c r="G21" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I21" s="8" t="s">
+      <c r="I21" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J21" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K21" s="8" t="s">
+      <c r="J21" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K21" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G22" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H22" s="8" t="s">
+      <c r="G22" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H22" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I22" s="8" t="s">
+      <c r="I22" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J22" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K22" s="8" t="s">
+      <c r="J22" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K22" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="G23" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H23" s="9" t="s">
+      <c r="H23" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I23" s="9" t="s">
+      <c r="I23" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="J23" s="9" t="s">
+      <c r="J23" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="K23" s="9" t="s">
+      <c r="K23" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E24" s="8" t="s">
+      <c r="E24" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="G24" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H24" s="8" t="s">
+      <c r="G24" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H24" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="I24" s="8" t="s">
+      <c r="I24" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="J24" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K24" s="8" t="s">
+      <c r="J24" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K24" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E25" s="8" t="s">
+      <c r="E25" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="G25" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H25" s="8" t="s">
+      <c r="G25" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H25" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="I25" s="8" t="s">
+      <c r="I25" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="J25" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K25" s="8" t="s">
+      <c r="J25" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K25" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="G26" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="H26" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I26" s="9" t="s">
+      <c r="I26" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="J26" s="9" t="s">
+      <c r="J26" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="K26" s="9" t="s">
+      <c r="K26" s="5" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="F27" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="H27" s="9" t="s">
+      <c r="H27" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I27" s="9" t="s">
+      <c r="I27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="J27" s="9" t="s">
+      <c r="J27" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="K27" s="9" t="s">
+      <c r="K27" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="D28" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="E28" s="9" t="s">
+      <c r="E28" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F28" s="9" t="s">
+      <c r="F28" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G28" s="9" t="s">
+      <c r="G28" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="H28" s="9" t="s">
+      <c r="H28" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I28" s="9" t="s">
+      <c r="I28" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="J28" s="9" t="s">
+      <c r="J28" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="K28" s="9" t="s">
+      <c r="K28" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="E29" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="F29" s="10" t="s">
+      <c r="F29" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="G29" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H29" s="10" t="s">
+      <c r="G29" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H29" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="I29" s="10" t="s">
+      <c r="I29" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="J29" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="K29" s="10" t="s">
+      <c r="J29" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K29" s="6" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="E30" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="F30" s="10" t="s">
+      <c r="F30" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="G30" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H30" s="10" t="s">
+      <c r="G30" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="I30" s="10" t="s">
+      <c r="I30" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="J30" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="K30" s="10" t="s">
+      <c r="J30" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K30" s="6" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="D31" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="E31" s="9" t="s">
+      <c r="E31" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F31" s="9" t="s">
+      <c r="F31" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G31" s="9" t="s">
+      <c r="G31" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H31" s="9" t="s">
+      <c r="H31" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I31" s="9" t="s">
+      <c r="I31" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J31" s="9" t="s">
+      <c r="J31" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="K31" s="9" t="s">
+      <c r="K31" s="5" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="D32" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E32" s="8" t="s">
+      <c r="E32" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F32" s="8" t="s">
+      <c r="F32" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G32" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H32" s="8" t="s">
+      <c r="G32" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H32" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="I32" s="8" t="s">
+      <c r="I32" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="J32" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K32" s="8" t="s">
+      <c r="J32" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K32" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="8" t="s">
+      <c r="A33" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D33" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E33" s="8" t="s">
+      <c r="E33" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="F33" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G33" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H33" s="8" t="s">
+      <c r="G33" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H33" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="I33" s="8" t="s">
+      <c r="I33" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="J33" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K33" s="8" t="s">
+      <c r="J33" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K33" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="D34" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E34" s="8" t="s">
+      <c r="E34" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F34" s="8" t="s">
+      <c r="F34" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G34" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H34" s="8" t="s">
+      <c r="G34" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H34" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="I34" s="8" t="s">
+      <c r="I34" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="J34" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K34" s="8" t="s">
+      <c r="J34" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K34" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D35" s="8" t="s">
+      <c r="D35" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E35" s="8" t="s">
+      <c r="E35" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F35" s="8" t="s">
+      <c r="F35" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G35" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H35" s="8" t="s">
+      <c r="G35" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H35" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="I35" s="8" t="s">
+      <c r="I35" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="J35" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K35" s="8" t="s">
+      <c r="J35" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K35" s="4" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" s="8" t="s">
+      <c r="A36" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D36" s="8" t="s">
+      <c r="D36" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E36" s="8" t="s">
+      <c r="E36" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F36" s="8" t="s">
+      <c r="F36" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G36" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H36" s="8" t="s">
+      <c r="G36" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H36" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="I36" s="8" t="s">
+      <c r="I36" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="J36" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K36" s="8" t="s">
+      <c r="J36" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K36" s="4" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D37" s="9" t="s">
+      <c r="D37" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E37" s="9" t="s">
+      <c r="E37" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F37" s="9" t="s">
+      <c r="F37" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G37" s="9" t="s">
+      <c r="G37" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="H37" s="9" t="s">
+      <c r="H37" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I37" s="9" t="s">
+      <c r="I37" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="J37" s="9" t="s">
+      <c r="J37" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="K37" s="9" t="s">
+      <c r="K37" s="5" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
+      <c r="A38" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B38" s="9" t="s">
+      <c r="B38" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="C38" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="D38" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="E38" s="9" t="s">
+      <c r="E38" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="F38" s="9" t="s">
+      <c r="F38" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G38" s="9" t="s">
+      <c r="G38" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="H38" s="9" t="s">
+      <c r="H38" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I38" s="9" t="s">
+      <c r="I38" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="J38" s="9" t="s">
+      <c r="J38" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="K38" s="9" t="s">
+      <c r="K38" s="5" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" s="10" t="s">
+      <c r="A39" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B39" s="10" t="s">
+      <c r="B39" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D39" s="10" t="s">
+      <c r="D39" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="E39" s="10" t="s">
+      <c r="E39" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="F39" s="10" t="s">
+      <c r="F39" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G39" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H39" s="10" t="s">
+      <c r="G39" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H39" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I39" s="10" t="s">
+      <c r="I39" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="J39" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="K39" s="10" t="s">
+      <c r="J39" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K39" s="6" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" s="10" t="s">
+      <c r="A40" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B40" s="10" t="s">
+      <c r="B40" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D40" s="10" t="s">
+      <c r="D40" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="E40" s="10" t="s">
+      <c r="E40" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="F40" s="10" t="s">
+      <c r="F40" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G40" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H40" s="10" t="s">
+      <c r="G40" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I40" s="10" t="s">
+      <c r="I40" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="J40" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="K40" s="10" t="s">
+      <c r="J40" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K40" s="6" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2153,7 +2156,7 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="1" max="1" width="25.42578125" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
@@ -2161,112 +2164,112 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="3" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="7" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="7" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="7" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="7" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2302,69 +2305,69 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
+      <c r="A2" s="10"/>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="10" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="10" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="14"/>
+      <c r="A6" s="10"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="10" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="10" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="10" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="10" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
+      <c r="A12" s="10"/>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="10" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="10" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
+      <c r="A15" s="10"/>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="10" t="s">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar Excel seguimiento con areas, registros y datos educacion completos
</commit_message>
<xml_diff>
--- a/ITT_Seguimiento_Datasets.xlsx
+++ b/ITT_Seguimiento_Datasets.xlsx
@@ -86,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -102,7 +102,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -471,20 +470,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: Mayo 2026 | - = Sin datos para ese trimestre</t>
+          <t>Generado: Mayo 2026 | - = Sin datos | ** = Proxy</t>
         </is>
       </c>
     </row>
@@ -509,50 +509,55 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>Area (m2)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
           <t>Dimension ITT</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Indicador</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Tipo Valor</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Score/Valor</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Periodo</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Formato</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -566,52 +571,57 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
           <t>Seguridad</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Homicidios</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>2023-2026 Q1</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>DATIC_homicidios_2023_2026T1_Barrio_O.geojson</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>3 registros total (2024-2025). Q2-Q4 2026 = -</t>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>3 registros (2024-2025). Q2-Q4 2026 = -</t>
         </is>
       </c>
     </row>
@@ -623,50 +633,55 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
           <t>Seguridad</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Hurtos</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>2023-2026 Q1</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>DATIC_hurtos_2023_2026T1_Barrio_O.geojson</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>155 registros. Q2-Q4 2026 = -</t>
         </is>
@@ -680,50 +695,55 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
           <t>Movilidad</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Siniestralidad</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>2023-2025</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>BD_SINIESTROS_2023_2025_COMUNA_BARRIO_OBRERO.geojson</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>15 registros. Sin datos 2026</t>
         </is>
@@ -737,50 +757,55 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
           <t>Movilidad</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Lesionados</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>2023-2025</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>BD_SINIESTROS (filtro Lesiones)</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Filtro Tipo_Confi=Lesiones</t>
         </is>
@@ -794,50 +819,55 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
           <t>Movilidad</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Mortales</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>2023-2025</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>BD_SINIESTROS (filtro Mortal)</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>Filtro Tipo_Confi=Mortal</t>
         </is>
@@ -851,52 +881,57 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
           <t>Entorno Urbano</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Deficit Habitacional</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Proxy</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>39.2 (o recalculado)</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>BD_DEFICIT_HABITACIONAL (Excel)</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>Excel</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>Proxy experimental con Comuna 9</t>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Proxy experimental Comuna 9</t>
         </is>
       </c>
     </row>
@@ -908,52 +943,57 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
           <t>Educacion</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Matricula</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>13%</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Proxy+Real</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>54.9 (2023-25) / 31.5 (2026)</t>
-        </is>
-      </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
+          <t>54.9 (23-25) / 31.5 (26)</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>geojson_educacion.zip + 01_Matricula_2026.xlsx</t>
-        </is>
-      </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>GeoJSON/Excel</t>
+          <t>geojson_educacion.zip</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Proxy 54.9 para 2023-2025. Real 31.5 para Q1 2026 (SIMAT, Comuna 9)</t>
+          <t>GeoJSON</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Proxy 54.9 para 2023-2025. Real 31.5 Q1 2026</t>
         </is>
       </c>
     </row>
@@ -965,52 +1005,57 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
           <t>Educacion</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Repitencia</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>13%</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>6.82%</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>SIMAT 2026</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>Excel</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>Constante municipal (no varia por comuna)</t>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>Constante municipal</t>
         </is>
       </c>
     </row>
@@ -1022,50 +1067,55 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
           <t>Educacion</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Est/Docente</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>13%</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Constante</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>24.64</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>SIMAT 2026</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>Excel</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>Constante municipal</t>
         </is>
@@ -1079,52 +1129,57 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
           <t>Educacion</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Est/Equipo</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>13%</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>22.3</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>03_Estudiantes_por_docente_y_equipo_2026.xlsx</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>Excel</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
-          <t>Agregado de sedes Comuna 9</t>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>Agregado sedes Comuna 9</t>
         </is>
       </c>
     </row>
@@ -1136,50 +1191,55 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
           <t>Cohesion Social</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>VIF</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>12%</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>2023-2026 Q1</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>DATIC_violencia_intrafamiliar_2023_2026T1_Barrio_O.geojson</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>24 registros. Q2-Q4 2026 = -</t>
         </is>
@@ -1193,52 +1253,57 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
           <t>Cohesion Social</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Rinas</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>12%</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>2023-2026 Q1</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>DATIC_comparendos_2023_2026T1_Barrio_O.geojson</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Filtro startswith(RI). Q2-Q4 2026 = -</t>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Filtro startswith(RI). 374 reg total</t>
         </is>
       </c>
     </row>
@@ -1250,50 +1315,55 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
           <t>Cohesion Social</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Vulnerabilidad</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>12%</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Proxy</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>54.1</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>Pulmon de Oriente</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="L16" s="5" t="inlineStr">
         <is>
           <t>Score fijo heredado</t>
         </is>
@@ -1307,50 +1377,55 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
+          <t>428,258</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
           <t>Seguridad</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Homicidios</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>2023-2025</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>HOMICIDIOS_2023_2025_Roosevelt.geojson</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>Datos reales</t>
         </is>
@@ -1364,50 +1439,55 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
+          <t>428,258</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
           <t>Seguridad</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Hurtos</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>2023-2025</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>HURTOS_2023_2025_Roosevelt.geojson</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>Datos reales</t>
         </is>
@@ -1421,677 +1501,737 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
+          <t>428,258</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
           <t>Movilidad</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Siniestralidad</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>2023-2025</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>BD_SINIESTROS_2023_2025_Roosevelt.geojson</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="L19" s="4" t="inlineStr">
         <is>
           <t>Datos reales</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Roosevelt</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>428,258</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Movilidad</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Lesionados</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>COMPLETA</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Calculado</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>2023-2025</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>BD_SINIESTROS (filtro Lesiones)</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>GeoJSON</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Datos reales</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Roosevelt</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>428,258</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Movilidad</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Mortales</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>COMPLETA</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Calculado</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>2023-2025</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>BD_SINIESTROS (filtro Mortal)</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>GeoJSON</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Datos reales</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Roosevelt</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>428,258</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Entorno Urbano</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Proxy</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>39.2</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>Pulmon de Oriente</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="L22" s="5" t="inlineStr">
         <is>
           <t>Score fijo heredado</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Roosevelt</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>428,258</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Educacion</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>13%</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>Proxy</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>54.9</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr">
         <is>
           <t>Pulmon de Oriente</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="K23" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="L23" s="5" t="inlineStr">
         <is>
           <t>Score fijo heredado</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Roosevelt</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>428,258</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Cohesion Social</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>VIF + Rinas</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>VIF</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>12%</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>2023-2025</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>VIF + COMPARENDOS Roosevelt</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>VIOLENCIA_INTRAFAMILIAR_2023_2025_Roosevelt.geojson</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>Vulnerabilidad: proxy 54.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Pulmon de Oriente</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Seguridad</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Homicidios + Hurtos</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Datos reales</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Roosevelt</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>428,258</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Cohesion Social</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Rinas</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Real+Proxy**</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>2023-2026 (Q2-Q4 Proxy**)</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>DATIC_*_Pulmon_O.geojson</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>2023-2025</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>COMPARENDOS_2023_2025_Roosevelt.geojson</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>Q2-Q4 2026 = Proxy**</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Pulmon de Oriente</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Movilidad</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>PROXY</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Proxy</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>35.0</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>Pulmon de Oriente</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>No hay siniestros en ZIP</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Pulmon de Oriente</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Entorno Urbano</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>PROXY</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>Proxy</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>39.2</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>Guia metodologica</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>Score fijo</t>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Filtro startswith(RI)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
+          <t>Roosevelt</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>428,258</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Cohesion Social</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Vulnerabilidad</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Proxy</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>54.1</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
           <t>Pulmon de Oriente</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Educacion</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="K26" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>13%</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>PROXY</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Proxy</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>54.9</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>Guia metodologica</t>
-        </is>
-      </c>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K26" s="5" t="inlineStr">
-        <is>
-          <t>Score fijo</t>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>Score fijo heredado</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Pulmon de Oriente</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Cohesion Social</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>VIF + Rinas</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>12%</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>5,503,953</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Homicidios</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>COMPLETA</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>Real+Proxy**</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>2023-2026 (Q2-Q4 Proxy**)</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>DATIC_*_Pulmon_O.geojson</t>
-        </is>
-      </c>
-      <c r="J27" s="6" t="inlineStr">
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>DATIC_homicidios_2023_2026T1_Pulmon_O.geojson</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K27" s="6" t="inlineStr">
-        <is>
-          <t>Vulnerabilidad: proxy 54.1</t>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Q1 real. Q2-Q4 = Proxy**</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Av. Ciudad de Cali</t>
+          <t>Pulmon de Oriente</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
+          <t>5,503,953</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
           <t>Seguridad</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Homicidios + Hurtos</t>
-        </is>
-      </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
+          <t>Hurtos</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>COMPLETA*</t>
-        </is>
-      </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Real</t>
+          <t>COMPLETA</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
+          <t>Real+Proxy**</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>2023-2025</t>
-        </is>
-      </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>GeoJSON (no versionado)</t>
+          <t>2023-2026 (Q2-Q4 Proxy**)</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
+          <t>DATIC_hurtos_2023_2026T1_Pulmon_O.geojson</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>*min-max relativo</t>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Q1 real. Q2-Q4 = Proxy**</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Av. Ciudad de Cali</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Pulmon de Oriente</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>5,503,953</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>Movilidad</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Siniestros</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>COMPLETA*</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Real</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>Calculado</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>2023-2025</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>GeoJSON (no versionado)</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>GeoJSON</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>*min-max relativo</t>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Proxy</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Pulmon de Oriente</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>No hay siniestros en ZIP</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Av. Ciudad de Cali</t>
+          <t>Pulmon de Oriente</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
+          <t>5,503,953</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
           <t>Entorno Urbano</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>Proxy</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>39.2</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="I30" s="5" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>Pulmon de Oriente</t>
-        </is>
-      </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
+          <t>Guia metodologica</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K30" s="5" t="inlineStr">
+      <c r="L30" s="5" t="inlineStr">
         <is>
           <t>Score fijo</t>
         </is>
@@ -2100,55 +2240,60 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Av. Ciudad de Cali</t>
+          <t>Pulmon de Oriente</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
+          <t>5,503,953</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
           <t>Educacion</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>13%</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>Proxy</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>54.9</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>Pulmon de Oriente</t>
-        </is>
-      </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
+          <t>Guia metodologica</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K31" s="5" t="inlineStr">
+      <c r="L31" s="5" t="inlineStr">
         <is>
           <t>Score fijo</t>
         </is>
@@ -2157,55 +2302,494 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
+          <t>Pulmon de Oriente</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>5,503,953</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Cohesion Social</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>VIF</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Real+Proxy**</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>Calculado</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>2023-2026 (Q2-Q4 Proxy**)</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>DATIC_violencia_intrafamiliar_2023_2026T1.geojson</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t>GeoJSON</t>
+        </is>
+      </c>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>Q1 real. Q2-Q4 = Proxy**</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Pulmon de Oriente</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>5,503,953</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Cohesion Social</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Rinas</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Real+Proxy**</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>Calculado</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>2023-2026 (Q2-Q4 Proxy**)</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>DATIC_comparendos_2023_2026T1_Pulmon_O.geojson</t>
+        </is>
+      </c>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>GeoJSON</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>Q1 real. Q2-Q4 = Proxy**</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Pulmon de Oriente</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>5,503,953</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Cohesion Social</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Vulnerabilidad</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Proxy</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>54.1</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>Sec. Bienestar Social</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>Score fijo heredado</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
           <t>Av. Ciudad de Cali</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Homicidios + Hurtos</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>COMPLETA*</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Calculado</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>2023-2025</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>GeoJSON (no versionado)</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>GeoJSON</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>*min-max relativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Av. Ciudad de Cali</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Movilidad</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Siniestros</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>COMPLETA*</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>Calculado</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>2023-2025</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>GeoJSON (no versionado)</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>GeoJSON</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>*min-max relativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Av. Ciudad de Cali</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Entorno Urbano</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Proxy</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>39.2</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>Pulmon de Oriente</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>Score fijo</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Av. Ciudad de Cali</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Educacion</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>13%</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>PROXY</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Proxy</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>54.9</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>Pulmon de Oriente</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>Score fijo</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Av. Ciudad de Cali</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Cohesion Social</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>VIF + Rinas</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>12%</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>Calculado</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="I39" s="6" t="inlineStr">
         <is>
           <t>2023-2025</t>
         </is>
       </c>
-      <c r="I32" s="6" t="inlineStr">
+      <c r="J39" s="6" t="inlineStr">
         <is>
           <t>GeoJSON (no versionado)</t>
         </is>
       </c>
-      <c r="J32" s="6" t="inlineStr">
+      <c r="K39" s="6" t="inlineStr">
         <is>
           <t>GeoJSON</t>
         </is>
       </c>
-      <c r="K32" s="6" t="inlineStr">
+      <c r="L39" s="6" t="inlineStr">
         <is>
           <t>Sin Vulnerabilidad</t>
         </is>
@@ -2213,8 +2797,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2226,7 +2810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2237,185 +2821,235 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Zona</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Area (m2)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Area (ha)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Seguridad</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Movilidad</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>Entorno Urbano</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Entorno U.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Educacion</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Cohesion</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Periodo</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Barrio Obrero</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>74,564</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>7.46</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>PARCIAL (54.9/31.5)</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>COMPLETA (Vuln=Proxy)</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>COMPLETA</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>2023-2026 Q1</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Roosevelt</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>428,258</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>42.83</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>PROXY (39.2)</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>PROXY (54.9)</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>COMPLETA (Vuln=Proxy)</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>COMPLETA</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>2023-2025</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Pulmon de Oriente</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>5,503,953</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>550.40</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>COMPLETA</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>PROXY (35.0)</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>PROXY (39.2)</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>PROXY (54.9)</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>2023-2026 (Proxy**)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Av. Ciudad de Cali</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>COMPLETA*</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>COMPLETA*</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>PROXY (39.2)</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>PROXY (54.9)</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>2023-2025</t>
         </is>
@@ -2432,7 +3066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -2451,35 +3085,35 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Barrio Obrero - Educacion:</t>
+          <t>Areas de poligonos (CRS: EPSG:3115 MAGNA-SIRGAS Colombia Oeste):</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2023-2025: Proxy 54.9 (Pulmon de Oriente, sin datos propios)</t>
+          <t xml:space="preserve">  Barrio Obrero: 74,564 m2 (7.46 ha) - Poligono unico</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2026 Q1: Real 31.5 (SIMAT 2026, Comuna 9)</t>
+          <t xml:space="preserve">  Roosevelt: 428,258 m2 (42.83 ha) - Corredor buffer 100m</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Indicadores: Matricula (6,561), Repitencia (6.82%), Est/Docente (24.64), Est/Equipo (22.3)</t>
+          <t xml:space="preserve">  Pulmon de Oriente: 5,503,953 m2 (550.40 ha) - Zona agregada</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Fuente: geojson_educacion.zip + 01_Matricula_2026.xlsx</t>
+          <t xml:space="preserve">  Av. Ciudad de Cali: No calculada (datos no versionados)</t>
         </is>
       </c>
     </row>
@@ -2489,35 +3123,104 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Colores barras trimestrales (gradiente claro a oscuro):</t>
+          <t>Barrio Obrero - Educacion:</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Seguridad: #90CAF9, #42A5F5, #1565C0, #003366 (azul)</t>
+          <t xml:space="preserve">  2023-2025: Proxy 54.9 (Pulmon de Oriente)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Movilidad: #FFCC80, #FB8C00, #E65100, #4E2600 (naranja)</t>
+          <t xml:space="preserve">  2026 Q1: Real 31.5 (SIMAT 2026, Comuna 9)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Indicadores: Matricula (6,561), Repitencia (6.82%), Est/Docente (24.64), Est/Equipo (22.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Colores barras trimestrales (gradiente claro a oscuro):</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Seguridad: #90CAF9, #42A5F5, #1565C0, #003366 (azul)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Movilidad: #FFCC80, #FB8C00, #E65100, #4E2600 (naranja)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Cohesion: #CE93D8, #8E24AA, #4A148C, #1A0033 (purpura)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Educacion: #A5D6A7, #43A047, #1B5E20, #003300 (verde)</t>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Reglas:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - PROXY = valor no observado directamente (fijo heredado, promedio historico, experimental)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - COMPLETA = datos reales propios</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - PARCIAL = mezcla de datos reales + Proxy</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - ** = Proxy estimado (solo Pulmon de Oriente Q2-Q4 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - - = Sin datos para ese trimestre</t>
         </is>
       </c>
     </row>

</xml_diff>